<commit_message>
Fix tests and workflow env
</commit_message>
<xml_diff>
--- a/load-tests/reports/load-test-report.xlsx
+++ b/load-tests/reports/load-test-report.xlsx
@@ -27,7 +27,7 @@
     <t>Run Date</t>
   </si>
   <si>
-    <t>2026-10-29T16:32:40.651Z</t>
+    <t>2026-10-30T07:55:10.877Z</t>
   </si>
   <si>
     <t>Target Environment</t>
@@ -54,7 +54,7 @@
     <t>Requests Per Second (RPS)</t>
   </si>
   <si>
-    <t>780.23 req/s</t>
+    <t>488.05 req/s</t>
   </si>
   <si>
     <t>Failure Rate</t>
@@ -66,25 +66,25 @@
     <t>Average Latency</t>
   </si>
   <si>
-    <t>2.73 ms</t>
+    <t>71.32 ms</t>
   </si>
   <si>
     <t>Median (p50) Latency</t>
   </si>
   <si>
-    <t>2.48 ms</t>
+    <t>17.65 ms</t>
   </si>
   <si>
     <t>p90 Latency</t>
   </si>
   <si>
-    <t>4.72 ms</t>
+    <t>188.75 ms</t>
   </si>
   <si>
     <t>p95 Latency</t>
   </si>
   <si>
-    <t>5.92 ms</t>
+    <t>246.39 ms</t>
   </si>
   <si>
     <t>Minimum Latency</t>
@@ -96,7 +96,7 @@
     <t>Maximum Latency</t>
   </si>
   <si>
-    <t>170.43 ms</t>
+    <t>1663.53 ms</t>
   </si>
   <si>
     <t>Service Level Objectives &amp; Threshold Compliance</t>
@@ -174,7 +174,7 @@
     <t>/api/health</t>
   </si>
   <si>
-    <t>88.27</t>
+    <t>55.19</t>
   </si>
   <si>
     <t>/api/items?search={q}</t>
@@ -821,7 +821,7 @@
         <v>11</v>
       </c>
       <c r="C9" s="4">
-        <v>59584</v>
+        <v>37255</v>
       </c>
     </row>
     <row r="10" ht="20" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
@@ -1016,7 +1016,7 @@
         <v>52</v>
       </c>
       <c r="C2" s="11">
-        <v>6620</v>
+        <v>4139</v>
       </c>
       <c r="D2" s="11" t="s">
         <v>53</v>
@@ -1025,22 +1025,22 @@
         <v>15</v>
       </c>
       <c r="F2" s="11">
-        <v>0.5</v>
+        <v>36.99</v>
       </c>
       <c r="G2" s="11">
         <v>0</v>
       </c>
       <c r="H2" s="11">
-        <v>0.51</v>
+        <v>6.68</v>
       </c>
       <c r="I2" s="11">
-        <v>1.17</v>
+        <v>78.11</v>
       </c>
       <c r="J2" s="11">
-        <v>1.67</v>
+        <v>172.61</v>
       </c>
       <c r="K2" s="11">
-        <v>10.69</v>
+        <v>888.62</v>
       </c>
     </row>
     <row r="3" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
@@ -1051,7 +1051,7 @@
         <v>54</v>
       </c>
       <c r="C3" s="11">
-        <v>6620</v>
+        <v>4139</v>
       </c>
       <c r="D3" s="11" t="s">
         <v>53</v>
@@ -1060,22 +1060,22 @@
         <v>15</v>
       </c>
       <c r="F3" s="11">
-        <v>3.56</v>
+        <v>102.51</v>
       </c>
       <c r="G3" s="11">
-        <v>0.51</v>
+        <v>1.53</v>
       </c>
       <c r="H3" s="11">
-        <v>3.06</v>
+        <v>22.11</v>
       </c>
       <c r="I3" s="11">
-        <v>5.54</v>
+        <v>229.08</v>
       </c>
       <c r="J3" s="11">
-        <v>7.01</v>
+        <v>369.15</v>
       </c>
       <c r="K3" s="11">
-        <v>67.03</v>
+        <v>1507.4</v>
       </c>
     </row>
     <row r="4" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
@@ -1086,7 +1086,7 @@
         <v>55</v>
       </c>
       <c r="C4" s="11">
-        <v>6620</v>
+        <v>4139</v>
       </c>
       <c r="D4" s="11" t="s">
         <v>53</v>
@@ -1095,22 +1095,22 @@
         <v>15</v>
       </c>
       <c r="F4" s="11">
-        <v>3.54</v>
+        <v>80.74</v>
       </c>
       <c r="G4" s="11">
-        <v>0.51</v>
+        <v>1.51</v>
       </c>
       <c r="H4" s="11">
-        <v>3.1</v>
+        <v>21.73</v>
       </c>
       <c r="I4" s="11">
-        <v>5.47</v>
+        <v>201.05</v>
       </c>
       <c r="J4" s="11">
-        <v>6.97</v>
+        <v>246.3</v>
       </c>
       <c r="K4" s="11">
-        <v>60.25</v>
+        <v>1281.14</v>
       </c>
     </row>
     <row r="5" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
@@ -1121,7 +1121,7 @@
         <v>56</v>
       </c>
       <c r="C5" s="11">
-        <v>6620</v>
+        <v>4139</v>
       </c>
       <c r="D5" s="11" t="s">
         <v>53</v>
@@ -1130,22 +1130,22 @@
         <v>15</v>
       </c>
       <c r="F5" s="11">
-        <v>3.32</v>
+        <v>78.62</v>
       </c>
       <c r="G5" s="11">
-        <v>0.5</v>
+        <v>0.56</v>
       </c>
       <c r="H5" s="11">
-        <v>2.89</v>
+        <v>21.65</v>
       </c>
       <c r="I5" s="11">
-        <v>5.21</v>
+        <v>194.32</v>
       </c>
       <c r="J5" s="11">
-        <v>6.67</v>
+        <v>248.16</v>
       </c>
       <c r="K5" s="11">
-        <v>51.9</v>
+        <v>1037.71</v>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
@@ -1156,7 +1156,7 @@
         <v>57</v>
       </c>
       <c r="C6" s="11">
-        <v>6620</v>
+        <v>4139</v>
       </c>
       <c r="D6" s="11" t="s">
         <v>53</v>
@@ -1165,22 +1165,22 @@
         <v>15</v>
       </c>
       <c r="F6" s="11">
-        <v>3.82</v>
+        <v>114.66</v>
       </c>
       <c r="G6" s="11">
-        <v>0.5</v>
+        <v>1.04</v>
       </c>
       <c r="H6" s="11">
-        <v>3.2</v>
+        <v>27.3</v>
       </c>
       <c r="I6" s="11">
-        <v>6.25</v>
+        <v>280.88</v>
       </c>
       <c r="J6" s="11">
-        <v>8.24</v>
+        <v>443.8</v>
       </c>
       <c r="K6" s="11">
-        <v>21.42</v>
+        <v>1663.53</v>
       </c>
     </row>
     <row r="7" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
@@ -1191,7 +1191,7 @@
         <v>58</v>
       </c>
       <c r="C7" s="11">
-        <v>6620</v>
+        <v>4139</v>
       </c>
       <c r="D7" s="11" t="s">
         <v>53</v>
@@ -1200,22 +1200,22 @@
         <v>15</v>
       </c>
       <c r="F7" s="11">
-        <v>2.28</v>
+        <v>58.15</v>
       </c>
       <c r="G7" s="11">
-        <v>0</v>
+        <v>0.51</v>
       </c>
       <c r="H7" s="11">
-        <v>2.03</v>
+        <v>14.63</v>
       </c>
       <c r="I7" s="11">
-        <v>3.63</v>
+        <v>138.32</v>
       </c>
       <c r="J7" s="11">
-        <v>4.51</v>
+        <v>208.41</v>
       </c>
       <c r="K7" s="11">
-        <v>12.86</v>
+        <v>950.5</v>
       </c>
     </row>
     <row r="8" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
@@ -1226,7 +1226,7 @@
         <v>59</v>
       </c>
       <c r="C8" s="11">
-        <v>6620</v>
+        <v>4139</v>
       </c>
       <c r="D8" s="11" t="s">
         <v>53</v>
@@ -1235,22 +1235,22 @@
         <v>15</v>
       </c>
       <c r="F8" s="11">
-        <v>2.14</v>
+        <v>57.88</v>
       </c>
       <c r="G8" s="11">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="H8" s="11">
-        <v>1.85</v>
+        <v>14.26</v>
       </c>
       <c r="I8" s="11">
-        <v>3.47</v>
+        <v>140.93</v>
       </c>
       <c r="J8" s="11">
-        <v>4.42</v>
+        <v>207.8</v>
       </c>
       <c r="K8" s="11">
-        <v>57.68</v>
+        <v>932.46</v>
       </c>
     </row>
     <row r="9" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
@@ -1261,7 +1261,7 @@
         <v>60</v>
       </c>
       <c r="C9" s="11">
-        <v>6620</v>
+        <v>4139</v>
       </c>
       <c r="D9" s="11" t="s">
         <v>53</v>
@@ -1270,22 +1270,22 @@
         <v>15</v>
       </c>
       <c r="F9" s="11">
-        <v>3.51</v>
+        <v>61.12</v>
       </c>
       <c r="G9" s="11">
-        <v>0.5</v>
+        <v>1.27</v>
       </c>
       <c r="H9" s="11">
-        <v>3.19</v>
+        <v>16.2</v>
       </c>
       <c r="I9" s="11">
-        <v>5.19</v>
+        <v>139.57</v>
       </c>
       <c r="J9" s="11">
-        <v>6.14</v>
+        <v>211.35</v>
       </c>
       <c r="K9" s="11">
-        <v>170.43</v>
+        <v>1071.15</v>
       </c>
     </row>
     <row r="10" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
@@ -1296,7 +1296,7 @@
         <v>61</v>
       </c>
       <c r="C10" s="11">
-        <v>6620</v>
+        <v>4139</v>
       </c>
       <c r="D10" s="11" t="s">
         <v>53</v>
@@ -1305,22 +1305,22 @@
         <v>15</v>
       </c>
       <c r="F10" s="11">
-        <v>1.86</v>
+        <v>51.26</v>
       </c>
       <c r="G10" s="11">
-        <v>0</v>
+        <v>0.51</v>
       </c>
       <c r="H10" s="11">
-        <v>1.54</v>
+        <v>13.64</v>
       </c>
       <c r="I10" s="11">
-        <v>3.11</v>
+        <v>125.35</v>
       </c>
       <c r="J10" s="11">
-        <v>4.09</v>
+        <v>167.88</v>
       </c>
       <c r="K10" s="11">
-        <v>14.52</v>
+        <v>919.55</v>
       </c>
     </row>
   </sheetData>
@@ -1374,16 +1374,16 @@
         <v>50</v>
       </c>
       <c r="C2" s="11">
-        <v>1986</v>
+        <v>1242</v>
       </c>
       <c r="D2" s="11">
-        <v>397.2</v>
+        <v>248.4</v>
       </c>
       <c r="E2" s="11">
-        <v>2.91</v>
+        <v>76.12</v>
       </c>
       <c r="F2" s="11">
-        <v>6.4</v>
+        <v>266.29</v>
       </c>
       <c r="G2" s="11" t="s">
         <v>15</v>
@@ -1397,16 +1397,16 @@
         <v>100</v>
       </c>
       <c r="C3" s="11">
-        <v>3972</v>
+        <v>2484</v>
       </c>
       <c r="D3" s="11">
-        <v>794.4</v>
+        <v>496.8</v>
       </c>
       <c r="E3" s="11">
-        <v>2.93</v>
+        <v>76.51</v>
       </c>
       <c r="F3" s="11">
-        <v>6.44</v>
+        <v>267.9</v>
       </c>
       <c r="G3" s="11" t="s">
         <v>15</v>
@@ -1420,16 +1420,16 @@
         <v>100</v>
       </c>
       <c r="C4" s="11">
-        <v>3972</v>
+        <v>2484</v>
       </c>
       <c r="D4" s="11">
-        <v>794.4</v>
+        <v>496.8</v>
       </c>
       <c r="E4" s="11">
-        <v>2.76</v>
+        <v>72.13</v>
       </c>
       <c r="F4" s="11">
-        <v>6</v>
+        <v>249.73</v>
       </c>
       <c r="G4" s="11" t="s">
         <v>15</v>
@@ -1443,16 +1443,16 @@
         <v>100</v>
       </c>
       <c r="C5" s="11">
-        <v>3972</v>
+        <v>2484</v>
       </c>
       <c r="D5" s="11">
-        <v>794.4</v>
+        <v>496.8</v>
       </c>
       <c r="E5" s="11">
-        <v>2.56</v>
+        <v>67</v>
       </c>
       <c r="F5" s="11">
-        <v>5.49</v>
+        <v>228.49</v>
       </c>
       <c r="G5" s="11" t="s">
         <v>15</v>
@@ -1466,16 +1466,16 @@
         <v>100</v>
       </c>
       <c r="C6" s="11">
-        <v>3972</v>
+        <v>2484</v>
       </c>
       <c r="D6" s="11">
-        <v>794.4</v>
+        <v>496.8</v>
       </c>
       <c r="E6" s="11">
-        <v>2.52</v>
+        <v>65.85</v>
       </c>
       <c r="F6" s="11">
-        <v>5.38</v>
+        <v>223.71</v>
       </c>
       <c r="G6" s="11" t="s">
         <v>15</v>
@@ -1489,16 +1489,16 @@
         <v>100</v>
       </c>
       <c r="C7" s="11">
-        <v>3972</v>
+        <v>2484</v>
       </c>
       <c r="D7" s="11">
-        <v>794.4</v>
+        <v>496.8</v>
       </c>
       <c r="E7" s="11">
-        <v>2.67</v>
+        <v>69.73</v>
       </c>
       <c r="F7" s="11">
-        <v>5.76</v>
+        <v>239.78</v>
       </c>
       <c r="G7" s="11" t="s">
         <v>15</v>
@@ -1512,16 +1512,16 @@
         <v>100</v>
       </c>
       <c r="C8" s="11">
-        <v>3972</v>
+        <v>2484</v>
       </c>
       <c r="D8" s="11">
-        <v>794.4</v>
+        <v>496.8</v>
       </c>
       <c r="E8" s="11">
-        <v>2.87</v>
+        <v>75.07</v>
       </c>
       <c r="F8" s="11">
-        <v>6.29</v>
+        <v>261.93</v>
       </c>
       <c r="G8" s="11" t="s">
         <v>15</v>
@@ -1535,16 +1535,16 @@
         <v>100</v>
       </c>
       <c r="C9" s="11">
-        <v>3972</v>
+        <v>2484</v>
       </c>
       <c r="D9" s="11">
-        <v>794.4</v>
+        <v>496.8</v>
       </c>
       <c r="E9" s="11">
-        <v>2.95</v>
+        <v>76.96</v>
       </c>
       <c r="F9" s="11">
-        <v>6.48</v>
+        <v>269.79</v>
       </c>
       <c r="G9" s="11" t="s">
         <v>15</v>
@@ -1558,16 +1558,16 @@
         <v>100</v>
       </c>
       <c r="C10" s="11">
-        <v>3972</v>
+        <v>2484</v>
       </c>
       <c r="D10" s="11">
-        <v>794.4</v>
+        <v>496.8</v>
       </c>
       <c r="E10" s="11">
-        <v>2.82</v>
+        <v>73.67</v>
       </c>
       <c r="F10" s="11">
-        <v>6.15</v>
+        <v>256.14</v>
       </c>
       <c r="G10" s="11" t="s">
         <v>15</v>
@@ -1581,16 +1581,16 @@
         <v>100</v>
       </c>
       <c r="C11" s="11">
-        <v>3972</v>
+        <v>2484</v>
       </c>
       <c r="D11" s="11">
-        <v>794.4</v>
+        <v>496.8</v>
       </c>
       <c r="E11" s="11">
-        <v>2.61</v>
+        <v>68.22</v>
       </c>
       <c r="F11" s="11">
-        <v>5.61</v>
+        <v>233.52</v>
       </c>
       <c r="G11" s="11" t="s">
         <v>15</v>
@@ -1604,16 +1604,16 @@
         <v>100</v>
       </c>
       <c r="C12" s="11">
-        <v>3972</v>
+        <v>2484</v>
       </c>
       <c r="D12" s="11">
-        <v>794.4</v>
+        <v>496.8</v>
       </c>
       <c r="E12" s="11">
-        <v>2.51</v>
+        <v>65.61</v>
       </c>
       <c r="F12" s="11">
-        <v>5.35</v>
+        <v>222.74</v>
       </c>
       <c r="G12" s="11" t="s">
         <v>15</v>
@@ -1627,16 +1627,16 @@
         <v>100</v>
       </c>
       <c r="C13" s="11">
-        <v>3972</v>
+        <v>2484</v>
       </c>
       <c r="D13" s="11">
-        <v>794.4</v>
+        <v>496.8</v>
       </c>
       <c r="E13" s="11">
-        <v>2.61</v>
+        <v>68.26</v>
       </c>
       <c r="F13" s="11">
-        <v>5.62</v>
+        <v>233.7</v>
       </c>
       <c r="G13" s="11" t="s">
         <v>15</v>
@@ -1650,16 +1650,16 @@
         <v>100</v>
       </c>
       <c r="C14" s="11">
-        <v>3972</v>
+        <v>2484</v>
       </c>
       <c r="D14" s="11">
-        <v>794.4</v>
+        <v>496.8</v>
       </c>
       <c r="E14" s="11">
-        <v>2.82</v>
+        <v>73.72</v>
       </c>
       <c r="F14" s="11">
-        <v>6.16</v>
+        <v>256.33</v>
       </c>
       <c r="G14" s="11" t="s">
         <v>15</v>
@@ -1673,16 +1673,16 @@
         <v>100</v>
       </c>
       <c r="C15" s="11">
-        <v>3972</v>
+        <v>2484</v>
       </c>
       <c r="D15" s="11">
-        <v>794.4</v>
+        <v>496.8</v>
       </c>
       <c r="E15" s="11">
-        <v>2.95</v>
+        <v>76.97</v>
       </c>
       <c r="F15" s="11">
-        <v>6.48</v>
+        <v>269.82</v>
       </c>
       <c r="G15" s="11" t="s">
         <v>15</v>
@@ -1696,16 +1696,16 @@
         <v>20</v>
       </c>
       <c r="C16" s="11">
-        <v>794</v>
+        <v>497</v>
       </c>
       <c r="D16" s="11">
-        <v>158.8</v>
+        <v>99.4</v>
       </c>
       <c r="E16" s="11">
-        <v>2.87</v>
+        <v>75.03</v>
       </c>
       <c r="F16" s="11">
-        <v>6.29</v>
+        <v>261.77</v>
       </c>
       <c r="G16" s="11" t="s">
         <v>15</v>

</xml_diff>

<commit_message>
resolved selenium empty excel sheets issue
</commit_message>
<xml_diff>
--- a/load-tests/reports/load-test-report.xlsx
+++ b/load-tests/reports/load-test-report.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="84">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="131" uniqueCount="86">
   <si>
     <t>RentCart API Performance Load Test — Executive Summary</t>
   </si>
@@ -27,13 +27,19 @@
     <t>Run Date</t>
   </si>
   <si>
-    <t>2026-10-30T07:55:10.877Z</t>
+    <t>2026-10-30T09:05:25.688Z</t>
   </si>
   <si>
     <t>Target Environment</t>
   </si>
   <si>
     <t>http://localhost:4000</t>
+  </si>
+  <si>
+    <t>Execution Platform</t>
+  </si>
+  <si>
+    <t>k6 v0.54.0 on Windows 10.0.26300 (x64)</t>
   </si>
   <si>
     <t>Virtual Users (VUs)</t>
@@ -757,7 +763,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="B2:F24"/>
+  <dimension ref="B2:F25"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="4" customWidth="1"/>
@@ -820,16 +826,16 @@
       <c r="B9" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="C9" s="4">
-        <v>37255</v>
+      <c r="C9" s="3" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="10" ht="20" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B10" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="C10" s="4" t="s">
         <v>13</v>
+      </c>
+      <c r="C10" s="4">
+        <v>37255</v>
       </c>
     </row>
     <row r="11" ht="20" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
@@ -844,7 +850,7 @@
       <c r="B12" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="C12" s="3" t="s">
+      <c r="C12" s="4" t="s">
         <v>17</v>
       </c>
     </row>
@@ -888,55 +894,49 @@
         <v>27</v>
       </c>
     </row>
-    <row r="20" ht="26" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B20" s="5" t="s">
+    <row r="18" ht="20" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B18" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="C20" s="5"/>
-      <c r="D20" s="5"/>
-      <c r="E20" s="5"/>
-      <c r="F20" s="5"/>
-    </row>
-    <row r="21" ht="22" customHeight="1" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B21" s="6" t="s">
+      <c r="C18" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="C21" s="6" t="s">
+    </row>
+    <row r="21" ht="26" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B21" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="D21" s="6" t="s">
+      <c r="C21" s="5"/>
+      <c r="D21" s="5"/>
+      <c r="E21" s="5"/>
+      <c r="F21" s="5"/>
+    </row>
+    <row r="22" ht="22" customHeight="1" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B22" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="E21" s="6" t="s">
+      <c r="C22" s="6" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="22" ht="20" customHeight="1" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B22" s="7" t="s">
+      <c r="D22" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="C22" s="8" t="s">
+      <c r="E22" s="6" t="s">
         <v>34</v>
-      </c>
-      <c r="D22" s="7" t="s">
-        <v>15</v>
-      </c>
-      <c r="E22" s="9" t="s">
-        <v>35</v>
       </c>
     </row>
     <row r="23" ht="20" customHeight="1" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B23" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="C23" s="8" t="s">
         <v>36</v>
       </c>
-      <c r="C23" s="8" t="s">
+      <c r="D23" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="E23" s="9" t="s">
         <v>37</v>
-      </c>
-      <c r="D23" s="7" t="s">
-        <v>23</v>
-      </c>
-      <c r="E23" s="9" t="s">
-        <v>35</v>
       </c>
     </row>
     <row r="24" ht="20" customHeight="1" spans="2:5" x14ac:dyDescent="0.25">
@@ -947,16 +947,30 @@
         <v>39</v>
       </c>
       <c r="D24" s="7" t="s">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="E24" s="9" t="s">
-        <v>35</v>
+        <v>37</v>
+      </c>
+    </row>
+    <row r="25" ht="20" customHeight="1" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B25" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="C25" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="D25" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="E25" s="9" t="s">
+        <v>37</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="B2:F2"/>
-    <mergeCell ref="B20:F20"/>
+    <mergeCell ref="B21:F21"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
@@ -975,54 +989,54 @@
   <sheetData>
     <row r="1" ht="26" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="C1" s="10" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="D1" s="10" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="E1" s="10" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="F1" s="10" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="G1" s="10" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="H1" s="10" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="I1" s="10" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="J1" s="10" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="K1" s="10" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
     </row>
     <row r="2" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" s="11" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="B2" s="12" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="C2" s="11">
         <v>4139</v>
       </c>
       <c r="D2" s="11" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="E2" s="11" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="F2" s="11">
         <v>36.99</v>
@@ -1045,19 +1059,19 @@
     </row>
     <row r="3" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" s="11" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="B3" s="12" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="C3" s="11">
         <v>4139</v>
       </c>
       <c r="D3" s="11" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="E3" s="11" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="F3" s="11">
         <v>102.51</v>
@@ -1080,19 +1094,19 @@
     </row>
     <row r="4" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" s="11" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="B4" s="12" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="C4" s="11">
         <v>4139</v>
       </c>
       <c r="D4" s="11" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="E4" s="11" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="F4" s="11">
         <v>80.74</v>
@@ -1115,19 +1129,19 @@
     </row>
     <row r="5" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" s="11" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="B5" s="12" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C5" s="11">
         <v>4139</v>
       </c>
       <c r="D5" s="11" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="E5" s="11" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="F5" s="11">
         <v>78.62</v>
@@ -1150,19 +1164,19 @@
     </row>
     <row r="6" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" s="11" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="B6" s="12" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="C6" s="11">
         <v>4139</v>
       </c>
       <c r="D6" s="11" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="E6" s="11" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="F6" s="11">
         <v>114.66</v>
@@ -1185,19 +1199,19 @@
     </row>
     <row r="7" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" s="11" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="B7" s="12" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="C7" s="11">
         <v>4139</v>
       </c>
       <c r="D7" s="11" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="E7" s="11" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="F7" s="11">
         <v>58.15</v>
@@ -1220,19 +1234,19 @@
     </row>
     <row r="8" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" s="11" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="B8" s="12" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="C8" s="11">
         <v>4139</v>
       </c>
       <c r="D8" s="11" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="E8" s="11" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="F8" s="11">
         <v>57.88</v>
@@ -1255,19 +1269,19 @@
     </row>
     <row r="9" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" s="11" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="B9" s="12" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="C9" s="11">
         <v>4139</v>
       </c>
       <c r="D9" s="11" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="E9" s="11" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="F9" s="11">
         <v>61.12</v>
@@ -1290,19 +1304,19 @@
     </row>
     <row r="10" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" s="11" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="B10" s="12" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="C10" s="11">
         <v>4139</v>
       </c>
       <c r="D10" s="11" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="E10" s="11" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="F10" s="11">
         <v>51.26</v>
@@ -1345,30 +1359,30 @@
   <sheetData>
     <row r="1" ht="26" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="C1" s="10" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="D1" s="10" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="E1" s="10" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="F1" s="10" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="G1" s="10" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
     </row>
     <row r="2" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="11" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="B2" s="11">
         <v>50</v>
@@ -1386,12 +1400,12 @@
         <v>266.29</v>
       </c>
       <c r="G2" s="11" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
     </row>
     <row r="3" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="11" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="B3" s="11">
         <v>100</v>
@@ -1409,12 +1423,12 @@
         <v>267.9</v>
       </c>
       <c r="G3" s="11" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
     </row>
     <row r="4" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="11" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="B4" s="11">
         <v>100</v>
@@ -1432,12 +1446,12 @@
         <v>249.73</v>
       </c>
       <c r="G4" s="11" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
     </row>
     <row r="5" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="11" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="B5" s="11">
         <v>100</v>
@@ -1455,12 +1469,12 @@
         <v>228.49</v>
       </c>
       <c r="G5" s="11" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="11" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="B6" s="11">
         <v>100</v>
@@ -1478,12 +1492,12 @@
         <v>223.71</v>
       </c>
       <c r="G6" s="11" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
     </row>
     <row r="7" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="11" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="B7" s="11">
         <v>100</v>
@@ -1501,12 +1515,12 @@
         <v>239.78</v>
       </c>
       <c r="G7" s="11" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
     </row>
     <row r="8" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="11" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="B8" s="11">
         <v>100</v>
@@ -1524,12 +1538,12 @@
         <v>261.93</v>
       </c>
       <c r="G8" s="11" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
     </row>
     <row r="9" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="11" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B9" s="11">
         <v>100</v>
@@ -1547,12 +1561,12 @@
         <v>269.79</v>
       </c>
       <c r="G9" s="11" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
     </row>
     <row r="10" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="11" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="B10" s="11">
         <v>100</v>
@@ -1570,12 +1584,12 @@
         <v>256.14</v>
       </c>
       <c r="G10" s="11" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
     </row>
     <row r="11" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="11" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="B11" s="11">
         <v>100</v>
@@ -1593,12 +1607,12 @@
         <v>233.52</v>
       </c>
       <c r="G11" s="11" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
     </row>
     <row r="12" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="11" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="B12" s="11">
         <v>100</v>
@@ -1616,12 +1630,12 @@
         <v>222.74</v>
       </c>
       <c r="G12" s="11" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
     </row>
     <row r="13" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="11" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B13" s="11">
         <v>100</v>
@@ -1639,12 +1653,12 @@
         <v>233.7</v>
       </c>
       <c r="G13" s="11" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
     </row>
     <row r="14" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="11" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="B14" s="11">
         <v>100</v>
@@ -1662,12 +1676,12 @@
         <v>256.33</v>
       </c>
       <c r="G14" s="11" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
     </row>
     <row r="15" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="11" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="B15" s="11">
         <v>100</v>
@@ -1685,12 +1699,12 @@
         <v>269.82</v>
       </c>
       <c r="G15" s="11" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
     </row>
     <row r="16" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="11" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="B16" s="11">
         <v>20</v>
@@ -1708,7 +1722,7 @@
         <v>261.77</v>
       </c>
       <c r="G16" s="11" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
     </row>
   </sheetData>

</xml_diff>